<commit_message>
Code changes are done at office in 28-11-25
</commit_message>
<xml_diff>
--- a/src/test/resources/ImportTemplate/Pushdown.xlsx
+++ b/src/test/resources/ImportTemplate/Pushdown.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\ImportTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B694DA9-91BC-4D7B-A657-D4189BB148BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACBF3400-F5C5-4F09-89BF-02A79A130075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,10 +33,10 @@
     <t>sourceSql</t>
   </si>
   <si>
-    <t>SELECT * FROM public.STAFF</t>
+    <t>Pushdown_ImportSQL-DB-PostgreSQL--Customer</t>
   </si>
   <si>
-    <t>Pushdown_ImportSQL-DB--STAFF--</t>
+    <t>SELECT * FROM public.Customer</t>
   </si>
 </sst>
 </file>
@@ -367,7 +367,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -380,10 +380,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>